<commit_message>
Updated to allow all pandas period options
</commit_message>
<xml_diff>
--- a/mock_data/mock_IT_workflow_data.xlsx
+++ b/mock_data/mock_IT_workflow_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zachj\Documents\ZenQMS_Metrics\mock_data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zachj\Documents\My_Git_Projects\Workflow_Metric_Reporting\mock_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFBAF786-160D-456B-AECF-8777E36EE93F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A14506AB-5A14-465F-8066-E4885E7FB2D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23430" yWindow="3735" windowWidth="16200" windowHeight="9360" xr2:uid="{CC4F641A-4D62-4460-9232-5940B0063984}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{CC4F641A-4D62-4460-9232-5940B0063984}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="105">
   <si>
     <t>Workflow ID</t>
   </si>
@@ -348,13 +348,16 @@
   </si>
   <si>
     <t>Endpoint patch verification</t>
+  </si>
+  <si>
+    <t>Original Completed Datetime</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -366,6 +369,13 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="7"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -391,7 +401,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -405,11 +415,30 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="22" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="5">
+  <dxfs count="6">
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="7"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="27" formatCode="m/d/yyyy\ h:mm"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="27" formatCode="m/d/yyyy\ h:mm"/>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -457,13 +486,16 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F3DF2B75-268C-4D30-A85B-85242E0BB9ED}" name="Table1" displayName="Table1" ref="A1:D51" totalsRowShown="0" headerRowDxfId="4">
-  <autoFilter ref="A1:D51" xr:uid="{F3DF2B75-268C-4D30-A85B-85242E0BB9ED}"/>
-  <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{7A372AC1-32F5-49AE-B16D-419F07923553}" name="Workflow ID" dataDxfId="3"/>
-    <tableColumn id="2" xr3:uid="{FC0DFAB6-C035-44B0-B3AE-84F9F535BF10}" name="Workflow Description" dataDxfId="2"/>
-    <tableColumn id="3" xr3:uid="{AD90E39F-3739-4025-933C-07550B1E7F62}" name="Start Datetime" dataDxfId="1"/>
-    <tableColumn id="4" xr3:uid="{8E737371-6B99-4A63-9CB5-3D231402B7A6}" name="Completed Datetime" dataDxfId="0"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F3DF2B75-268C-4D30-A85B-85242E0BB9ED}" name="Table1" displayName="Table1" ref="A1:E51" totalsRowShown="0" headerRowDxfId="5">
+  <autoFilter ref="A1:E51" xr:uid="{F3DF2B75-268C-4D30-A85B-85242E0BB9ED}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{7A372AC1-32F5-49AE-B16D-419F07923553}" name="Workflow ID" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{FC0DFAB6-C035-44B0-B3AE-84F9F535BF10}" name="Workflow Description" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{AD90E39F-3739-4025-933C-07550B1E7F62}" name="Start Datetime" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{050577BC-EC45-43E9-BD13-FA3B1E288779}" name="Completed Datetime" dataDxfId="0">
+      <calculatedColumnFormula>Table1[[#This Row],[Start Datetime]]+(14*RAND())</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="4" xr3:uid="{8E737371-6B99-4A63-9CB5-3D231402B7A6}" name="Original Completed Datetime" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -786,15 +818,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{461C03C6-2172-43CC-90ED-BA1C3D70066D}">
-  <dimension ref="A1:D51"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:E51"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="12.28515625" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" customWidth="1"/>
-    <col min="3" max="4" width="19.140625" customWidth="1"/>
+    <col min="1" max="1" width="12.265625" customWidth="1"/>
+    <col min="2" max="2" width="30.3984375" customWidth="1"/>
+    <col min="3" max="5" width="19.1328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -807,8 +839,11 @@
       <c r="D1" s="3" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1" s="3" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -818,11 +853,15 @@
       <c r="C2" s="2">
         <v>45778.341666666667</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2" s="5">
+        <f ca="1">Table1[[#This Row],[Start Datetime]]+(14*RAND())</f>
+        <v>45787.478411053133</v>
+      </c>
+      <c r="E2" s="2">
         <v>45778.350694444445</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
@@ -832,11 +871,15 @@
       <c r="C3" s="2">
         <v>45778.375</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3" s="5">
+        <f ca="1">Table1[[#This Row],[Start Datetime]]+(14*RAND())</f>
+        <v>45786.431197756981</v>
+      </c>
+      <c r="E3" s="2">
         <v>45778.438888888886</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
@@ -846,11 +889,15 @@
       <c r="C4" s="2">
         <v>45778.597222222219</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="5">
+        <f ca="1">Table1[[#This Row],[Start Datetime]]+(14*RAND())</f>
+        <v>45784.585830396187</v>
+      </c>
+      <c r="E4" s="2">
         <v>45778.604861111111</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
         <v>10</v>
       </c>
@@ -860,11 +907,15 @@
       <c r="C5" s="2">
         <v>45779.28125</v>
       </c>
-      <c r="D5" s="2">
+      <c r="D5" s="5">
+        <f ca="1">Table1[[#This Row],[Start Datetime]]+(14*RAND())</f>
+        <v>45783.104310903684</v>
+      </c>
+      <c r="E5" s="2">
         <v>45779.329861111109</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
         <v>12</v>
       </c>
@@ -874,11 +925,15 @@
       <c r="C6" s="2">
         <v>45779.461805555555</v>
       </c>
-      <c r="D6" s="2">
+      <c r="D6" s="5">
+        <f ca="1">Table1[[#This Row],[Start Datetime]]+(14*RAND())</f>
+        <v>45791.54740287015</v>
+      </c>
+      <c r="E6" s="2">
         <v>45779.488888888889</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
         <v>14</v>
       </c>
@@ -888,11 +943,15 @@
       <c r="C7" s="2">
         <v>45779.631944444445</v>
       </c>
-      <c r="D7" s="2">
+      <c r="D7" s="5">
+        <f ca="1">Table1[[#This Row],[Start Datetime]]+(14*RAND())</f>
+        <v>45786.419737135351</v>
+      </c>
+      <c r="E7" s="2">
         <v>45779.643055555556</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
         <v>16</v>
       </c>
@@ -902,11 +961,15 @@
       <c r="C8" s="2">
         <v>45780.333333333336</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D8" s="5">
+        <f ca="1">Table1[[#This Row],[Start Datetime]]+(14*RAND())</f>
+        <v>45789.945273448757</v>
+      </c>
+      <c r="E8" s="2">
         <v>45780.359027777777</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A9" s="1" t="s">
         <v>18</v>
       </c>
@@ -916,11 +979,15 @@
       <c r="C9" s="2">
         <v>45780.552083333336</v>
       </c>
-      <c r="D9" s="2">
+      <c r="D9" s="5">
+        <f ca="1">Table1[[#This Row],[Start Datetime]]+(14*RAND())</f>
+        <v>45785.61977525874</v>
+      </c>
+      <c r="E9" s="2">
         <v>45780.577777777777</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A10" s="1" t="s">
         <v>20</v>
       </c>
@@ -930,11 +997,15 @@
       <c r="C10" s="2">
         <v>45780.673611111109</v>
       </c>
-      <c r="D10" s="2">
+      <c r="D10" s="5">
+        <f ca="1">Table1[[#This Row],[Start Datetime]]+(14*RAND())</f>
+        <v>45785.661312305987</v>
+      </c>
+      <c r="E10" s="2">
         <v>45780.7</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A11" s="1" t="s">
         <v>22</v>
       </c>
@@ -944,11 +1015,15 @@
       <c r="C11" s="2">
         <v>45781.390277777777</v>
       </c>
-      <c r="D11" s="2">
+      <c r="D11" s="5">
+        <f ca="1">Table1[[#This Row],[Start Datetime]]+(14*RAND())</f>
+        <v>45795.040061968226</v>
+      </c>
+      <c r="E11" s="2">
         <v>45781.397916666669</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A12" s="1" t="s">
         <v>24</v>
       </c>
@@ -958,11 +1033,15 @@
       <c r="C12" s="2">
         <v>45781.444444444445</v>
       </c>
-      <c r="D12" s="2">
+      <c r="D12" s="5">
+        <f ca="1">Table1[[#This Row],[Start Datetime]]+(14*RAND())</f>
+        <v>45789.410158922306</v>
+      </c>
+      <c r="E12" s="2">
         <v>45781.477777777778</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A13" s="1" t="s">
         <v>26</v>
       </c>
@@ -972,11 +1051,15 @@
       <c r="C13" s="2">
         <v>45781.583333333336</v>
       </c>
-      <c r="D13" s="2">
+      <c r="D13" s="5">
+        <f ca="1">Table1[[#This Row],[Start Datetime]]+(14*RAND())</f>
+        <v>45793.744413875225</v>
+      </c>
+      <c r="E13" s="2">
         <v>45781.621527777781</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A14" s="1" t="s">
         <v>28</v>
       </c>
@@ -986,11 +1069,15 @@
       <c r="C14" s="2">
         <v>45782.345833333333</v>
       </c>
-      <c r="D14" s="2">
+      <c r="D14" s="5">
+        <f ca="1">Table1[[#This Row],[Start Datetime]]+(14*RAND())</f>
+        <v>45791.529424161999</v>
+      </c>
+      <c r="E14" s="2">
         <v>45782.356944444444</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A15" s="1" t="s">
         <v>30</v>
       </c>
@@ -1000,11 +1087,15 @@
       <c r="C15" s="2">
         <v>45782.405555555553</v>
       </c>
-      <c r="D15" s="2">
+      <c r="D15" s="5">
+        <f ca="1">Table1[[#This Row],[Start Datetime]]+(14*RAND())</f>
+        <v>45794.413584361369</v>
+      </c>
+      <c r="E15" s="2">
         <v>45782.42291666667</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A16" s="1" t="s">
         <v>32</v>
       </c>
@@ -1014,11 +1105,15 @@
       <c r="C16" s="2">
         <v>45782.480555555558</v>
       </c>
-      <c r="D16" s="2">
+      <c r="D16" s="5">
+        <f ca="1">Table1[[#This Row],[Start Datetime]]+(14*RAND())</f>
+        <v>45783.107991364333</v>
+      </c>
+      <c r="E16" s="2">
         <v>45782.506944444445</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A17" s="1" t="s">
         <v>34</v>
       </c>
@@ -1028,11 +1123,15 @@
       <c r="C17" s="2">
         <v>45783.298611111109</v>
       </c>
-      <c r="D17" s="2">
+      <c r="D17" s="5">
+        <f ca="1">Table1[[#This Row],[Start Datetime]]+(14*RAND())</f>
+        <v>45794.258508870204</v>
+      </c>
+      <c r="E17" s="2">
         <v>45783.322916666664</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A18" s="1" t="s">
         <v>36</v>
       </c>
@@ -1042,11 +1141,15 @@
       <c r="C18" s="2">
         <v>45783.576388888891</v>
       </c>
-      <c r="D18" s="2">
+      <c r="D18" s="5">
+        <f ca="1">Table1[[#This Row],[Start Datetime]]+(14*RAND())</f>
+        <v>45792.81754511578</v>
+      </c>
+      <c r="E18" s="2">
         <v>45783.597222222219</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A19" s="1" t="s">
         <v>38</v>
       </c>
@@ -1056,11 +1159,15 @@
       <c r="C19" s="2">
         <v>45783.642361111109</v>
       </c>
-      <c r="D19" s="2">
+      <c r="D19" s="5">
+        <f ca="1">Table1[[#This Row],[Start Datetime]]+(14*RAND())</f>
+        <v>45793.264448801172</v>
+      </c>
+      <c r="E19" s="2">
         <v>45783.668749999997</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A20" s="1" t="s">
         <v>40</v>
       </c>
@@ -1070,11 +1177,15 @@
       <c r="C20" s="2">
         <v>45784.336805555555</v>
       </c>
-      <c r="D20" s="2">
+      <c r="D20" s="5">
+        <f ca="1">Table1[[#This Row],[Start Datetime]]+(14*RAND())</f>
+        <v>45789.19469073962</v>
+      </c>
+      <c r="E20" s="2">
         <v>45784.36041666667</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A21" s="1" t="s">
         <v>42</v>
       </c>
@@ -1084,11 +1195,15 @@
       <c r="C21" s="2">
         <v>45784.416666666664</v>
       </c>
-      <c r="D21" s="2">
+      <c r="D21" s="5">
+        <f ca="1">Table1[[#This Row],[Start Datetime]]+(14*RAND())</f>
+        <v>45786.554082718256</v>
+      </c>
+      <c r="E21" s="2">
         <v>45784.466666666667</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A22" s="1" t="s">
         <v>44</v>
       </c>
@@ -1098,11 +1213,15 @@
       <c r="C22" s="2">
         <v>45784.59375</v>
       </c>
-      <c r="D22" s="2">
+      <c r="D22" s="5">
+        <f ca="1">Table1[[#This Row],[Start Datetime]]+(14*RAND())</f>
+        <v>45791.790248314152</v>
+      </c>
+      <c r="E22" s="2">
         <v>45784.619444444441</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A23" s="1" t="s">
         <v>46</v>
       </c>
@@ -1112,11 +1231,15 @@
       <c r="C23" s="2">
         <v>45785.324999999997</v>
       </c>
-      <c r="D23" s="2">
+      <c r="D23" s="5">
+        <f ca="1">Table1[[#This Row],[Start Datetime]]+(14*RAND())</f>
+        <v>45793.146407679509</v>
+      </c>
+      <c r="E23" s="2">
         <v>45785.332638888889</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A24" s="1" t="s">
         <v>48</v>
       </c>
@@ -1126,11 +1249,15 @@
       <c r="C24" s="2">
         <v>45785.388888888891</v>
       </c>
-      <c r="D24" s="2">
+      <c r="D24" s="5">
+        <f ca="1">Table1[[#This Row],[Start Datetime]]+(14*RAND())</f>
+        <v>45797.264093164726</v>
+      </c>
+      <c r="E24" s="2">
         <v>45785.418055555558</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A25" s="1" t="s">
         <v>50</v>
       </c>
@@ -1140,11 +1267,15 @@
       <c r="C25" s="2">
         <v>45785.5625</v>
       </c>
-      <c r="D25" s="2">
+      <c r="D25" s="5">
+        <f ca="1">Table1[[#This Row],[Start Datetime]]+(14*RAND())</f>
+        <v>45793.491084390611</v>
+      </c>
+      <c r="E25" s="2">
         <v>45785.588194444441</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A26" s="1" t="s">
         <v>52</v>
       </c>
@@ -1154,11 +1285,15 @@
       <c r="C26" s="2">
         <v>45786.288194444445</v>
       </c>
-      <c r="D26" s="2">
+      <c r="D26" s="5">
+        <f ca="1">Table1[[#This Row],[Start Datetime]]+(14*RAND())</f>
+        <v>45796.01366381027</v>
+      </c>
+      <c r="E26" s="2">
         <v>45786.320138888892</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A27" s="1" t="s">
         <v>54</v>
       </c>
@@ -1168,11 +1303,15 @@
       <c r="C27" s="2">
         <v>45786.510416666664</v>
       </c>
-      <c r="D27" s="2">
+      <c r="D27" s="5">
+        <f ca="1">Table1[[#This Row],[Start Datetime]]+(14*RAND())</f>
+        <v>45800.28220172174</v>
+      </c>
+      <c r="E27" s="2">
         <v>45786.53125</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A28" s="1" t="s">
         <v>56</v>
       </c>
@@ -1182,11 +1321,15 @@
       <c r="C28" s="2">
         <v>45786.631944444445</v>
       </c>
-      <c r="D28" s="2">
+      <c r="D28" s="5">
+        <f ca="1">Table1[[#This Row],[Start Datetime]]+(14*RAND())</f>
+        <v>45790.416972432533</v>
+      </c>
+      <c r="E28" s="2">
         <v>45786.670138888891</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A29" s="1" t="s">
         <v>58</v>
       </c>
@@ -1196,11 +1339,15 @@
       <c r="C29" s="2">
         <v>45787.355555555558</v>
       </c>
-      <c r="D29" s="2">
+      <c r="D29" s="5">
+        <f ca="1">Table1[[#This Row],[Start Datetime]]+(14*RAND())</f>
+        <v>45800.010511747525</v>
+      </c>
+      <c r="E29" s="2">
         <v>45787.387499999997</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A30" s="1" t="s">
         <v>60</v>
       </c>
@@ -1210,11 +1357,15 @@
       <c r="C30" s="2">
         <v>45787.473611111112</v>
       </c>
-      <c r="D30" s="2">
+      <c r="D30" s="5">
+        <f ca="1">Table1[[#This Row],[Start Datetime]]+(14*RAND())</f>
+        <v>45797.145775524972</v>
+      </c>
+      <c r="E30" s="2">
         <v>45787.493750000001</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A31" s="1" t="s">
         <v>62</v>
       </c>
@@ -1224,11 +1375,15 @@
       <c r="C31" s="2">
         <v>45787.612500000003</v>
       </c>
-      <c r="D31" s="2">
+      <c r="D31" s="5">
+        <f ca="1">Table1[[#This Row],[Start Datetime]]+(14*RAND())</f>
+        <v>45798.574912897704</v>
+      </c>
+      <c r="E31" s="2">
         <v>45787.629861111112</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A32" s="1" t="s">
         <v>64</v>
       </c>
@@ -1238,11 +1393,15 @@
       <c r="C32" s="2">
         <v>45788.375</v>
       </c>
-      <c r="D32" s="2">
+      <c r="D32" s="5">
+        <f ca="1">Table1[[#This Row],[Start Datetime]]+(14*RAND())</f>
+        <v>45792.829276772602</v>
+      </c>
+      <c r="E32" s="2">
         <v>45788.387499999997</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A33" s="1" t="s">
         <v>66</v>
       </c>
@@ -1252,11 +1411,15 @@
       <c r="C33" s="2">
         <v>45788.4375</v>
       </c>
-      <c r="D33" s="2">
+      <c r="D33" s="5">
+        <f ca="1">Table1[[#This Row],[Start Datetime]]+(14*RAND())</f>
+        <v>45800.962454100656</v>
+      </c>
+      <c r="E33" s="2">
         <v>45788.472222222219</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A34" s="1" t="s">
         <v>68</v>
       </c>
@@ -1266,11 +1429,15 @@
       <c r="C34" s="2">
         <v>45788.569444444445</v>
       </c>
-      <c r="D34" s="2">
+      <c r="D34" s="5">
+        <f ca="1">Table1[[#This Row],[Start Datetime]]+(14*RAND())</f>
+        <v>45800.260115430814</v>
+      </c>
+      <c r="E34" s="2">
         <v>45788.584722222222</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A35" s="1" t="s">
         <v>70</v>
       </c>
@@ -1280,11 +1447,15 @@
       <c r="C35" s="2">
         <v>45789.301388888889</v>
       </c>
-      <c r="D35" s="2">
+      <c r="D35" s="5">
+        <f ca="1">Table1[[#This Row],[Start Datetime]]+(14*RAND())</f>
+        <v>45791.640296907761</v>
+      </c>
+      <c r="E35" s="2">
         <v>45789.322916666664</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A36" s="1" t="s">
         <v>72</v>
       </c>
@@ -1294,11 +1465,15 @@
       <c r="C36" s="2">
         <v>45789.534722222219</v>
       </c>
-      <c r="D36" s="2">
+      <c r="D36" s="5">
+        <f ca="1">Table1[[#This Row],[Start Datetime]]+(14*RAND())</f>
+        <v>45796.404618606895</v>
+      </c>
+      <c r="E36" s="2">
         <v>45789.55972222222</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A37" s="1" t="s">
         <v>74</v>
       </c>
@@ -1308,11 +1483,15 @@
       <c r="C37" s="2">
         <v>45789.673611111109</v>
       </c>
-      <c r="D37" s="2">
+      <c r="D37" s="5">
+        <f ca="1">Table1[[#This Row],[Start Datetime]]+(14*RAND())</f>
+        <v>45798.830246075864</v>
+      </c>
+      <c r="E37" s="2">
         <v>45789.686111111114</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A38" s="1" t="s">
         <v>76</v>
       </c>
@@ -1322,11 +1501,15 @@
       <c r="C38" s="2">
         <v>45790.350694444445</v>
       </c>
-      <c r="D38" s="2">
+      <c r="D38" s="5">
+        <f ca="1">Table1[[#This Row],[Start Datetime]]+(14*RAND())</f>
+        <v>45798.921034392391</v>
+      </c>
+      <c r="E38" s="2">
         <v>45790.370833333334</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A39" s="1" t="s">
         <v>78</v>
       </c>
@@ -1336,11 +1519,15 @@
       <c r="C39" s="2">
         <v>45790.486111111109</v>
       </c>
-      <c r="D39" s="2">
+      <c r="D39" s="5">
+        <f ca="1">Table1[[#This Row],[Start Datetime]]+(14*RAND())</f>
+        <v>45802.234192579817</v>
+      </c>
+      <c r="E39" s="2">
         <v>45790.51458333333</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A40" s="1" t="s">
         <v>80</v>
       </c>
@@ -1350,11 +1537,15 @@
       <c r="C40" s="2">
         <v>45790.625</v>
       </c>
-      <c r="D40" s="2">
+      <c r="D40" s="5">
+        <f ca="1">Table1[[#This Row],[Start Datetime]]+(14*RAND())</f>
+        <v>45803.369551348063</v>
+      </c>
+      <c r="E40" s="2">
         <v>45790.649305555555</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A41" s="1" t="s">
         <v>82</v>
       </c>
@@ -1364,11 +1555,15 @@
       <c r="C41" s="2">
         <v>45791.390277777777</v>
       </c>
-      <c r="D41" s="2">
+      <c r="D41" s="5">
+        <f ca="1">Table1[[#This Row],[Start Datetime]]+(14*RAND())</f>
+        <v>45804.291801182844</v>
+      </c>
+      <c r="E41" s="2">
         <v>45791.40902777778</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A42" s="1" t="s">
         <v>84</v>
       </c>
@@ -1378,11 +1573,15 @@
       <c r="C42" s="2">
         <v>45791.465277777781</v>
       </c>
-      <c r="D42" s="2">
+      <c r="D42" s="5">
+        <f ca="1">Table1[[#This Row],[Start Datetime]]+(14*RAND())</f>
+        <v>45798.296900779424</v>
+      </c>
+      <c r="E42" s="2">
         <v>45791.505555555559</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A43" s="1" t="s">
         <v>86</v>
       </c>
@@ -1392,11 +1591,15 @@
       <c r="C43" s="2">
         <v>45791.618055555555</v>
       </c>
-      <c r="D43" s="2">
+      <c r="D43" s="5">
+        <f ca="1">Table1[[#This Row],[Start Datetime]]+(14*RAND())</f>
+        <v>45797.716297721054</v>
+      </c>
+      <c r="E43" s="2">
         <v>45791.64166666667</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A44" s="1" t="s">
         <v>88</v>
       </c>
@@ -1406,11 +1609,15 @@
       <c r="C44" s="2">
         <v>45792.3125</v>
       </c>
-      <c r="D44" s="2">
+      <c r="D44" s="5">
+        <f ca="1">Table1[[#This Row],[Start Datetime]]+(14*RAND())</f>
+        <v>45799.342535132069</v>
+      </c>
+      <c r="E44" s="2">
         <v>45792.334722222222</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A45" s="1" t="s">
         <v>90</v>
       </c>
@@ -1420,11 +1627,15 @@
       <c r="C45" s="2">
         <v>45792.430555555555</v>
       </c>
-      <c r="D45" s="2">
+      <c r="D45" s="5">
+        <f ca="1">Table1[[#This Row],[Start Datetime]]+(14*RAND())</f>
+        <v>45805.690048910976</v>
+      </c>
+      <c r="E45" s="2">
         <v>45792.44027777778</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A46" s="1" t="s">
         <v>92</v>
       </c>
@@ -1434,11 +1645,15 @@
       <c r="C46" s="2">
         <v>45792.670138888891</v>
       </c>
-      <c r="D46" s="2">
+      <c r="D46" s="5">
+        <f ca="1">Table1[[#This Row],[Start Datetime]]+(14*RAND())</f>
+        <v>45804.386163856354</v>
+      </c>
+      <c r="E46" s="2">
         <v>45792.686805555553</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A47" s="1" t="s">
         <v>94</v>
       </c>
@@ -1448,11 +1663,15 @@
       <c r="C47" s="2">
         <v>45793.375</v>
       </c>
-      <c r="D47" s="2">
+      <c r="D47" s="5">
+        <f ca="1">Table1[[#This Row],[Start Datetime]]+(14*RAND())</f>
+        <v>45806.993878768815</v>
+      </c>
+      <c r="E47" s="2">
         <v>45793.411805555559</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A48" s="1" t="s">
         <v>96</v>
       </c>
@@ -1462,11 +1681,15 @@
       <c r="C48" s="2">
         <v>45793.475694444445</v>
       </c>
-      <c r="D48" s="2">
+      <c r="D48" s="5">
+        <f ca="1">Table1[[#This Row],[Start Datetime]]+(14*RAND())</f>
+        <v>45805.967445802366</v>
+      </c>
+      <c r="E48" s="2">
         <v>45793.506944444445</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A49" s="1" t="s">
         <v>98</v>
       </c>
@@ -1476,11 +1699,15 @@
       <c r="C49" s="2">
         <v>45793.595833333333</v>
       </c>
-      <c r="D49" s="2">
+      <c r="D49" s="5">
+        <f ca="1">Table1[[#This Row],[Start Datetime]]+(14*RAND())</f>
+        <v>45802.919229873958</v>
+      </c>
+      <c r="E49" s="2">
         <v>45793.599999999999</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A50" s="1" t="s">
         <v>100</v>
       </c>
@@ -1490,11 +1717,15 @@
       <c r="C50" s="2">
         <v>45794.322916666664</v>
       </c>
-      <c r="D50" s="2">
+      <c r="D50" s="5">
+        <f ca="1">Table1[[#This Row],[Start Datetime]]+(14*RAND())</f>
+        <v>45796.714478107897</v>
+      </c>
+      <c r="E50" s="2">
         <v>45794.36041666667</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A51" s="1" t="s">
         <v>102</v>
       </c>
@@ -1504,7 +1735,11 @@
       <c r="C51" s="2">
         <v>45794.465277777781</v>
       </c>
-      <c r="D51" s="2">
+      <c r="D51" s="5">
+        <f ca="1">Table1[[#This Row],[Start Datetime]]+(14*RAND())</f>
+        <v>45808.294761539888</v>
+      </c>
+      <c r="E51" s="2">
         <v>45794.486111111109</v>
       </c>
     </row>

</xml_diff>